<commit_message>
fix(seeds): one row each so MAX(id) returns non-NULL in sequence resets
bcgov's migration e15dc8fa858a does `SELECT MAX(id) INTO maxid` then
`ALTER SEQUENCE … RESTART WITH maxid+1`. On an empty table MAX(id) is
NULL and NULL+1 is NULL, breaking the EXECUTE. One row per seed file
makes MAX(id) at least 1.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/api/alembic/seeds/Languages.xlsx
+++ b/api/alembic/seeds/Languages.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -423,6 +423,13 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>